<commit_message>
Refocus Day 28 lab on P-047 safety monitoring
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -15,10 +15,10 @@
     <sheet name="Change_Log" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Metrics'!$A$1:$J$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflow'!$A$1:$F$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Metrics'!$A$1:$J$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Workflow'!$A$1:$F$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Roadmap_30_60_90'!$A$1:$F$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Evidence'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Evidence'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Change_Log'!$A$1:$D$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -203,12 +203,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Metrics'!$B$2:$B$6</f>
+              <f>'Metrics'!$B$2:$B$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Metrics'!$C$2:$C$6</f>
+              <f>'Metrics'!$C$2:$C$7</f>
             </numRef>
           </val>
         </ser>
@@ -227,12 +227,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Metrics'!$B$2:$B$6</f>
+              <f>'Metrics'!$B$2:$B$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Metrics'!$D$2:$D$6</f>
+              <f>'Metrics'!$D$2:$D$7</f>
             </numRef>
           </val>
         </ser>
@@ -267,7 +267,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Giá trị</a:t>
+                  <a:t>Giá trị (xem đơn vị trong sheet Metrics)</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -293,10 +293,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>10</row>
+      <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5400000" cy="2520000"/>
+    <ext cx="6480000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -603,17 +603,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DASHBOARD HÀNH ĐỘNG ÁP DỤNG AI — V2</t>
+          <t>DASHBOARD HÀNH ĐỘNG ÁP DỤNG AI — P-047 — V2</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Trợ lý AI tra cứu quy định và tài liệu nội bộ có trích nguồn</t>
+          <t>P-047 Safety Monitoring — Computer Vision giám sát PPE và vùng cấm</t>
         </is>
       </c>
     </row>
@@ -637,11 +637,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nhân viên vận hành mới trong 90 ngày đầu</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>Safety Manager; System Admin; Area Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Quy trình</t>
@@ -649,7 +649,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tiếp nhận → truy xuất → trả lời có nguồn → xác nhận/chuyển tuyến</t>
+          <t>Upload/gán media → cấu hình rule → inference/cảnh báo → HITL/audit</t>
         </is>
       </c>
     </row>
@@ -661,22 +661,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SỬA rồi tiếp tục pilot có kiểm soát</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n"/>
+          <t>SỬA trước khi pilot; chưa rollout nhà máy</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Lưu ý dữ liệu</t>
+          <t>Nguồn</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Số liệu pilot mô phỏng phục vụ bài lab; phải thay bằng log thật trước khi tuyên bố tác động.</t>
+          <t>P-047 revision c929e50; evidence 071c575; operational log đến 01/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Giới hạn</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Log là traffic phát triển/test; local DB có 0 safety event; US-13 chưa hoàn tất.</t>
         </is>
       </c>
     </row>
@@ -695,19 +704,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="37" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="53" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -770,14 +779,14 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Tỷ lệ hoàn thành tác vụ không cần hỏi lại</t>
+          <t>Tỷ lệ cảnh báo hữu ích được HITL xác nhận</t>
         </is>
       </c>
       <c r="C2" s="4" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
@@ -786,7 +795,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Event log + xác nhận outcome</t>
+          <t>safety_events status; baseline 0 đủ mẫu</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -801,31 +810,31 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Phân tích intent thất bại; sửa top 3 luồng</t>
+          <t>Dừng mở rộng; hiệu chỉnh model/rule và review false alarm</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>≥70% ngày 90</t>
+          <t>≥100 event hoặc ≥2 tuần pilot</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Product safety</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Tỷ lệ câu trả lời vượt QA nguồn</t>
+          <t>Recall tình huống critical trên ground truth</t>
         </is>
       </c>
       <c r="C3" s="4" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
@@ -834,27 +843,27 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Mẫu QA 30 câu/tuần</t>
+          <t>US-13 held-out evaluation; chưa đo</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Tuần</t>
+          <t>Mỗi model</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>QA Lead</t>
+          <t>Vision Lead</t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Dừng mở rộng; sửa nguồn/prompt trong 48h</t>
+          <t>Không pilot; bổ sung dữ liệu và hiệu chỉnh threshold</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>≥75% để qua gate ngày 60</t>
+          <t>≥95%, không bỏ sót Sev-1</t>
         </is>
       </c>
     </row>
@@ -866,14 +875,14 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Tỷ lệ yêu cầu xử lý trong SLA</t>
+          <t>Tỷ lệ inference hoàn thành</t>
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>55</v>
+        <v>78.2</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
@@ -882,128 +891,176 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Queue timestamps</t>
+          <t>1.544 completed / (1.544 + 430 failed)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Tuần</t>
+          <t>Ngày</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Knowledge Manager</t>
+          <t>Platform Owner</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Bổ sung owner hoặc giảm phạm vi nguồn</t>
+          <t>Phân loại error; rollback provider; kiểm tra health</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>≥85% ngày 60</t>
+          <t>Log dev/test, phải re-baseline pilot</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Guardrail</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Tỷ lệ chuyển tuyến đúng</t>
+          <t>P95 inference latency</t>
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>8</v>
+        <v>1306</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>15</v>
+        <v>1000</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>% tối đa</t>
+          <t>ms</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Escalation log</t>
+          <t>operational-metrics.jsonl</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Tuần</t>
+          <t>Ngày</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>AI Governance Lead</t>
+          <t>Vision Lead</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Nếu &gt;15%: rà coverage; nếu quá thấp: audit false confidence</t>
+          <t>Giảm FPS/tải; warm worker; chặn rollout nếu stale</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>≤15%, không có sự cố nghiêm trọng</t>
+          <t>E2E alert target ≤2.000 ms</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Activity</t>
+          <t>Quality gate</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Số câu hỏi/người/tuần</t>
+          <t>Backend/Vision tests pass</t>
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>3</v>
+        <v>95.59999999999999</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>câu tham khảo</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Event log</t>
+          <t>304 pass / 318; 14 known fail</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
+          <t>Theo PR</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>QA Lead</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Sửa hoặc phân loại; không còn Sev-1/2</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Bắt buộc trước pilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Guardrail</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Snapshot không lộ danh tính</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Manual MAN-04 + privacy fail-closed test</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>Tuần</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Adoption Lead</t>
-        </is>
-      </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>Dùng để chẩn đoán, không coi là giá trị</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Không dùng làm gate</t>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Privacy Owner</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Dừng lưu snapshot và điều tra ngay</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>0 privacy incident</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J6"/>
+  <autoFilter ref="A1:J7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1014,15 +1071,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1033,12 +1090,12 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>AS-IS</t>
+          <t>AS-IS hiện có</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>TO-BE</t>
+          <t>TO-BE sau chẩn đoán</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
@@ -1048,7 +1105,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>AI hỗ trợ/tự động</t>
+          <t>Vai trò AI</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -1063,27 +1120,27 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Gõ câu hỏi tự do</t>
+          <t>System Admin upload và gán asset</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Chọn loại câu hỏi + nhập bối cảnh</t>
+          <t>Kiểm tra provenance, quyền lưu và readiness trước khi gán</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Người dùng</t>
+          <t>System Admin</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>AI phân loại intent</t>
+          <t>AI chưa tham gia</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Không thu dữ liệu nhạy cảm</t>
+          <t>Media private; decode validation</t>
         </is>
       </c>
     </row>
@@ -1093,27 +1150,27 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>AI tìm trong kho không rõ độ mới</t>
+          <t>Safety Manager cấu hình PPE/vùng</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Truy xuất chỉ nguồn có owner, hiệu lực, quyền</t>
+          <t>Rule có owner, version, severity và escalation policy</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Knowledge Manager</t>
+          <t>Safety Manager</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>AI xếp hạng đoạn liên quan</t>
+          <t>AI áp rule deterministic</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Lọc quyền + freshness gate</t>
+          <t>Zone revision; role authorization</t>
         </is>
       </c>
     </row>
@@ -1123,27 +1180,27 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Trả lời có thể thiếu nguồn</t>
+          <t>AI detect/track và mở candidate</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Câu trả lời kèm nguồn, đoạn, ngày cập nhật</t>
+          <t>Ghi freshness, latency, model version; fail-closed khi lỗi</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Người dùng chịu trách nhiệm kết quả</t>
+          <t>Vision + Platform Owner</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>AI soạn nháp</t>
+          <t>AI tự động quan sát, không kết luận cuối</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Không đủ nguồn thì từ chối/chuyển tuyến</t>
+          <t>Debounce; dedup; health gate</t>
         </is>
       </c>
     </row>
@@ -1153,32 +1210,62 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Không ghi outcome</t>
+          <t>HITL xác nhận đúng/báo sai</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Đã giải quyết/chưa giải quyết + lý do</t>
+          <t>Thêm SLA review, reason code và queue escalation</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Product Owner</t>
+          <t>Safety Manager</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>AI gắn tag lỗi</t>
+          <t>AI trình bằng chứng đã làm mờ</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>QA mẫu + escalation queue</t>
+          <t>Privacy fail-closed; immutable audit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Area Manager xử lý event</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Theo dõi time-to-resolve và owner theo camera/khu vực</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Area Manager</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>AI tóm tắt chỉ mang tính hỗ trợ</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Area-scoped authorization</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F5"/>
+  <autoFilter ref="A1:F6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1193,11 +1280,11 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="57" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1240,27 +1327,27 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Chuẩn hóa nguồn và pilot hẹp</t>
+          <t>Tạo baseline đáng tin</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Gắn owner/SLA; dựng event log; đào tạo tại điểm dùng</t>
+          <t>Chốt provenance; ground truth US-13; browser UAT; xử lý 14 failure</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Knowledge Manager + Product Owner</t>
+          <t>Vision Lead + QA Lead</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>100% nguồn có metadata; 20 người pilot</t>
+          <t>≥200 scenario có nhãn; 0 blocker Sev-1/2</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Không có nguồn không owner</t>
+          <t>Chưa qua thì không pilot</t>
         </is>
       </c>
     </row>
@@ -1272,22 +1359,22 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Nâng chất lượng và khả năng</t>
+          <t>Pilot hẹp có HITL</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>QA 30 câu/tuần; sửa top lỗi; office hour</t>
+          <t>Một khu vực/một ca; đo precision, recall, false alarm, review SLA</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>QA Lead + Adoption Lead</t>
+          <t>Safety Manager + Product Owner</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>QA ≥75%; completion ≥65%</t>
+          <t>Precision ≥85%; critical recall ≥95%; review SLA ≥90%</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1309,7 +1396,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Mở thêm nhóm; theo dõi guardrail; review gate</t>
+          <t>Soak 4 camera/30 phút; privacy audit; escalation/rollback drill</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1319,7 +1406,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>QA ≥90%; completion ≥70%; SLA ≥85%</t>
+          <t>P95 alert ≤2s; 0 privacy incident; capacity report</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1340,20 +1427,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Loại</t>
+          <t>Nguồn</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -1363,103 +1450,157 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Quan sát</t>
+          <t>Kết quả có thật</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Kết quả</t>
+          <t>Dùng để kết luận</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Giới hạn</t>
+          <t>Không được suy diễn</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Pilot mô phỏng</t>
+          <t>Manual UI 01/09/2026</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>100 tác vụ</t>
+          <t>7 case</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Người dùng thử tra cứu theo checklist</t>
+          <t>7/7 PASS</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>42 tác vụ hoàn thành không hỏi lại</t>
+          <t>Luồng PPE, zone, HITL/privacy, auth, reconnect hoạt động</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Không đại diện doanh nghiệp thật</t>
+          <t>Không chứng minh accuracy nhà máy</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>QA nguồn mô phỏng</t>
+          <t>Focused backend 071c575</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>100 câu trả lời</t>
+          <t>11 checks</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra nguồn tồn tại, đúng đoạn, hiệu lực, quyền</t>
+          <t>11/11 PASS trong 3,03s</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>58 câu vượt QA</t>
+          <t>Zone threshold, privacy fail-closed, idempotency, authorization</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Cần QA độc lập với dữ liệu thật</t>
+          <t>Không đại diện full suite</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Queue mô phỏng</t>
+          <t>Quality gate rộng</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>100 yêu cầu</t>
+          <t>318 backend/vision</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>So timestamp tiếp nhận và xử lý</t>
+          <t>304 pass, 14 fail đã biết</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>55 yêu cầu trong SLA</t>
+          <t>Repo còn nợ chất lượng cần xử lý/phân loại</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>SLA cần thống nhất với owner thật</t>
+          <t>Không được báo toàn repo xanh</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Operational JSONL</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>12.292 record</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>1.544 completed; 430 failed; 834 dropped; P95 1.306ms</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Baseline kỹ thuật dev/test</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Không phải production KPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Local safety_events.db</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>0 event</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Chưa có outcome HITL đủ mẫu</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Baseline product hiện chưa đo</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Không bịa precision/false alarm</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:E6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1474,9 +1615,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="65" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -1507,17 +1648,17 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Số câu hỏi/người là metric đích</t>
+          <t>Dùng inference/event count làm metric adoption</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Đổi sang completion không cần hỏi lại; usage chỉ còn signal</t>
+          <t>Đổi sang alert usefulness, critical recall và review SLA</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>Đo giá trị thay vì hoạt động</t>
+          <t>Đo giá trị và an toàn thay vì activity</t>
         </is>
       </c>
     </row>
@@ -1527,17 +1668,17 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Có citation</t>
+          <t>Diễn giải 7/7 manual pass là sẵn sàng</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>QA citation theo tồn tại/đúng đoạn/hiệu lực/quyền + stop gate</t>
+          <t>Tách functional evidence khỏi US-13/pilot/capacity evidence</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Tăng độ tin cậy và khả năng hành động</t>
+          <t>Tránh kết luận vượt quá bằng chứng</t>
         </is>
       </c>
     </row>
@@ -1547,17 +1688,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Owner chưa tách rõ</t>
+          <t>Không có stop gate rõ</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Chỉ định Product, QA, Knowledge, Adoption, Governance owner</t>
+          <t>Thêm privacy, recall, precision, latency và severity gate theo owner</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Tránh coi AI là người chịu trách nhiệm</t>
+          <t>Mỗi chỉ số dẫn tới quyết định/hành động</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: make v1 and v2 review changes auditable
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -782,8 +782,10 @@
           <t>Tỷ lệ cảnh báo hữu ích được HITL xác nhận</t>
         </is>
       </c>
-      <c r="C2" s="4" t="n">
-        <v>0</v>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Chưa đo (0 event)</t>
+        </is>
       </c>
       <c r="D2" s="4" t="n">
         <v>85</v>
@@ -795,7 +797,7 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>safety_events status; baseline 0 đủ mẫu</t>
+          <t>safety_events: (acknowledged + resolved) / total reviewed</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -815,7 +817,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>≥100 event hoặc ≥2 tuần pilot</t>
+          <t>Chỉ lập baseline khi ≥100 event hoặc ≥2 tuần pilot</t>
         </is>
       </c>
     </row>
@@ -830,8 +832,10 @@
           <t>Recall tình huống critical trên ground truth</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Chưa đo (US-13 mở)</t>
+        </is>
       </c>
       <c r="D3" s="4" t="n">
         <v>95</v>
@@ -843,7 +847,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>US-13 held-out evaluation; chưa đo</t>
+          <t>US-13 held-out: true positive / total critical ground truth</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -1019,14 +1023,18 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Snapshot không lộ danh tính</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>100</v>
+          <t>Tỷ lệ snapshot vượt privacy audit</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>1/1 test PASS</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>100% mẫu pilot</t>
+        </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
@@ -1035,7 +1043,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Manual MAN-04 + privacy fail-closed test</t>
+          <t>Manual MAN-04 + privacy audit mẫu pilot</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -1055,7 +1063,7 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>0 privacy incident</t>
+          <t>0 privacy incident; chưa suy rộng từ 1 test</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1103,7 @@
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>TO-BE sau chẩn đoán</t>
+          <t>TO-BE</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">

</xml_diff>